<commit_message>
Changed Gain to Summary for Figure 10; Clarify population of worksheets
</commit_message>
<xml_diff>
--- a/figures/Figure 10/Gain_200K_real.xlsx
+++ b/figures/Figure 10/Gain_200K_real.xlsx
@@ -5,15 +5,15 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\prata\Files\Git\Causal-Search-for-Skylines\graphs\Figure 10\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\prata\Files\Git\Causal-Search-for-Skylines\figures\Figure 10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2913CEA3-8517-40E8-A8C9-3DF39957A553}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F6AAC5F-1639-4161-9F47-CA19C78A7C59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Gain" sheetId="1" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -852,7 +852,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Gain!$E$166</c:f>
+              <c:f>Summary!$E$166</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1062,11 +1062,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>Gain!$F$165:$K$165</c15:sqref>
+                    <c15:sqref>Summary!$F$165:$K$165</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(Gain!$F$165:$G$165,Gain!$K$165)</c:f>
+              <c:f>(Summary!$F$165:$G$165,Summary!$K$165)</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -1086,11 +1086,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>Gain!$F$166:$K$166</c15:sqref>
+                    <c15:sqref>Summary!$F$166:$K$166</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(Gain!$F$166:$G$166,Gain!$K$166)</c:f>
+              <c:f>(Summary!$F$166:$G$166,Summary!$K$166)</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -2500,13 +2500,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K167"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="7" width="10" customWidth="1"/>
     <col min="8" max="11" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.45">
       <c r="F1" s="7" t="s">
         <v>0</v>
       </c>
@@ -2516,7 +2516,7 @@
       <c r="J1" s="8"/>
       <c r="K1" s="8"/>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
       <c r="E2" s="5" t="s">
         <v>172</v>
       </c>
@@ -2539,7 +2539,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>21</v>
       </c>
@@ -2574,7 +2574,7 @@
         <v>24.44100754423998</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>21</v>
       </c>
@@ -2609,7 +2609,7 @@
         <v>24.383270713267851</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>21</v>
       </c>
@@ -2644,7 +2644,7 @@
         <v>23.339287880435581</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>21</v>
       </c>
@@ -2679,7 +2679,7 @@
         <v>24.344175413995981</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>21</v>
       </c>
@@ -2714,7 +2714,7 @@
         <v>23.333878052420911</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>21</v>
       </c>
@@ -2749,7 +2749,7 @@
         <v>23.401692059775819</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>21</v>
       </c>
@@ -2784,7 +2784,7 @@
         <v>24.464753385959192</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>21</v>
       </c>
@@ -2819,7 +2819,7 @@
         <v>24.51220761560835</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A11">
         <v>21</v>
       </c>
@@ -2854,7 +2854,7 @@
         <v>24.560424385359511</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A12">
         <v>21</v>
       </c>
@@ -2889,7 +2889,7 @@
         <v>24.42144146342762</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A13">
         <v>21</v>
       </c>
@@ -2924,7 +2924,7 @@
         <v>24.505366238020361</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A14">
         <v>21</v>
       </c>
@@ -2959,7 +2959,7 @@
         <v>23.34147017858923</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A15">
         <v>21</v>
       </c>
@@ -2994,7 +2994,7 @@
         <v>23.26154542057775</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A16">
         <v>21</v>
       </c>
@@ -3029,7 +3029,7 @@
         <v>23.27690991703421</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A17">
         <v>21</v>
       </c>
@@ -3064,7 +3064,7 @@
         <v>24.416344241192569</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A18">
         <v>21</v>
       </c>
@@ -3099,7 +3099,7 @@
         <v>23.37746360120364</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A19">
         <v>22</v>
       </c>
@@ -3134,7 +3134,7 @@
         <v>1.458216420700774</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A20">
         <v>22</v>
       </c>
@@ -3169,7 +3169,7 @@
         <v>1.474472042359412</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A21">
         <v>22</v>
       </c>
@@ -3204,7 +3204,7 @@
         <v>1.4385841960553081</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A22">
         <v>22</v>
       </c>
@@ -3239,7 +3239,7 @@
         <v>1.4500491374637929</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A23">
         <v>22</v>
       </c>
@@ -3274,7 +3274,7 @@
         <v>1.447367609012872</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A24">
         <v>22</v>
       </c>
@@ -3309,7 +3309,7 @@
         <v>1.4383837636094541</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A25">
         <v>22</v>
       </c>
@@ -3344,7 +3344,7 @@
         <v>1.458843974163756</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A26">
         <v>22</v>
       </c>
@@ -3379,7 +3379,7 @@
         <v>1.450301648164168</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A27">
         <v>23</v>
       </c>
@@ -3414,7 +3414,7 @@
         <v>0.1908992333803326</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A28">
         <v>23</v>
       </c>
@@ -3449,7 +3449,7 @@
         <v>0.19473268971778451</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A29">
         <v>23</v>
       </c>
@@ -3484,7 +3484,7 @@
         <v>0.1945206654723734</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A30">
         <v>23</v>
       </c>
@@ -3519,7 +3519,7 @@
         <v>0.19097568956203759</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A31">
         <v>23</v>
       </c>
@@ -3554,7 +3554,7 @@
         <v>0.19240865795873099</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A32">
         <v>23</v>
       </c>
@@ -3589,7 +3589,7 @@
         <v>0.19141147723421451</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A33">
         <v>23</v>
       </c>
@@ -3624,7 +3624,7 @@
         <v>0.191566958418116</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A34">
         <v>23</v>
       </c>
@@ -3659,7 +3659,7 @@
         <v>0.19502577683888381</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A35">
         <v>23</v>
       </c>
@@ -3694,7 +3694,7 @@
         <v>0.19366440940648319</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A36">
         <v>23</v>
       </c>
@@ -3729,7 +3729,7 @@
         <v>0.19318844983354211</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A37">
         <v>23</v>
       </c>
@@ -3764,7 +3764,7 @@
         <v>0.19172542416490609</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A38">
         <v>23</v>
       </c>
@@ -3799,7 +3799,7 @@
         <v>0.19097886034287509</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A39">
         <v>23</v>
       </c>
@@ -3834,7 +3834,7 @@
         <v>0.1933852895628661</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A40">
         <v>23</v>
       </c>
@@ -3869,7 +3869,7 @@
         <v>0.19258559234440331</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A41">
         <v>23</v>
       </c>
@@ -3904,7 +3904,7 @@
         <v>0.19832254298962651</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A42">
         <v>23</v>
       </c>
@@ -3939,7 +3939,7 @@
         <v>0.19105716738849879</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A43">
         <v>24</v>
       </c>
@@ -3974,7 +3974,7 @@
         <v>6.2385046621784568E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A44">
         <v>24</v>
       </c>
@@ -4009,7 +4009,7 @@
         <v>6.2136991182342172E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A45">
         <v>24</v>
       </c>
@@ -4044,7 +4044,7 @@
         <v>6.3067925628274679E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A46">
         <v>24</v>
       </c>
@@ -4079,7 +4079,7 @@
         <v>6.3343228679150348E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A47">
         <v>24</v>
       </c>
@@ -4114,7 +4114,7 @@
         <v>6.3011122960597271E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A48">
         <v>24</v>
       </c>
@@ -4149,7 +4149,7 @@
         <v>6.3678649161010986E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A49">
         <v>24</v>
       </c>
@@ -4184,7 +4184,7 @@
         <v>6.3199707353487608E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A50">
         <v>24</v>
       </c>
@@ -4219,7 +4219,7 @@
         <v>6.3047227403149012E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A51">
         <v>24</v>
       </c>
@@ -4254,7 +4254,7 @@
         <v>6.3320311438292268E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A52">
         <v>24</v>
       </c>
@@ -4289,7 +4289,7 @@
         <v>6.3518787128850812E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A53">
         <v>24</v>
       </c>
@@ -4324,7 +4324,7 @@
         <v>6.2687130598351362E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A54">
         <v>24</v>
       </c>
@@ -4359,7 +4359,7 @@
         <v>6.3301519816741342E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A55">
         <v>24</v>
       </c>
@@ -4394,7 +4394,7 @@
         <v>6.3998343003913757E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A56">
         <v>24</v>
       </c>
@@ -4429,7 +4429,7 @@
         <v>6.2632403802126646E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A57">
         <v>24</v>
       </c>
@@ -4464,7 +4464,7 @@
         <v>6.3882928341627121E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A58">
         <v>24</v>
       </c>
@@ -4499,7 +4499,7 @@
         <v>6.2991091003641489E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A59">
         <v>4</v>
       </c>
@@ -4534,7 +4534,7 @@
         <v>4.9735700245946653E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A60">
         <v>4</v>
       </c>
@@ -4569,7 +4569,7 @@
         <v>5.0725550809875133E-2</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A61">
         <v>4</v>
       </c>
@@ -4604,7 +4604,7 @@
         <v>5.0758045911788938E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A62">
         <v>4</v>
       </c>
@@ -4639,7 +4639,7 @@
         <v>5.1610156288370491E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A63">
         <v>4</v>
       </c>
@@ -4674,7 +4674,7 @@
         <v>4.9825186375528567E-2</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A64">
         <v>4</v>
       </c>
@@ -4709,7 +4709,7 @@
         <v>5.065844114869833E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A65">
         <v>4</v>
       </c>
@@ -4744,7 +4744,7 @@
         <v>4.9256567982956773E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A66">
         <v>4</v>
       </c>
@@ -4779,7 +4779,7 @@
         <v>5.0015226332470783E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A67">
         <v>5</v>
       </c>
@@ -4814,7 +4814,7 @@
         <v>0.47761725559830659</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A68">
         <v>5</v>
       </c>
@@ -4849,7 +4849,7 @@
         <v>0.4762780965305865</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A69">
         <v>5</v>
       </c>
@@ -4884,7 +4884,7 @@
         <v>0.47948132683522998</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A70">
         <v>5</v>
       </c>
@@ -4919,7 +4919,7 @@
         <v>0.47901779459789401</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A71">
         <v>5</v>
       </c>
@@ -4954,7 +4954,7 @@
         <v>0.49029234098270541</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A72">
         <v>5</v>
       </c>
@@ -4989,7 +4989,7 @@
         <v>0.48311937516555192</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A73">
         <v>5</v>
       </c>
@@ -5024,7 +5024,7 @@
         <v>0.47579807145521053</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A74">
         <v>5</v>
       </c>
@@ -5059,7 +5059,7 @@
         <v>0.48032507719472051</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A75">
         <v>5</v>
       </c>
@@ -5094,7 +5094,7 @@
         <v>0.48382840799167748</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A76">
         <v>5</v>
       </c>
@@ -5129,7 +5129,7 @@
         <v>0.48329052077606321</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A77">
         <v>5</v>
       </c>
@@ -5164,7 +5164,7 @@
         <v>0.4844450967386365</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A78">
         <v>5</v>
       </c>
@@ -5199,7 +5199,7 @@
         <v>0.47740822378546</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A79">
         <v>5</v>
       </c>
@@ -5234,7 +5234,7 @@
         <v>0.48560613724403079</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A80">
         <v>5</v>
       </c>
@@ -5269,7 +5269,7 @@
         <v>0.48326090257614851</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A81">
         <v>5</v>
       </c>
@@ -5304,7 +5304,7 @@
         <v>0.48280500881373878</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A82">
         <v>5</v>
       </c>
@@ -5339,7 +5339,7 @@
         <v>0.47904408997856079</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A83">
         <v>5</v>
       </c>
@@ -5374,7 +5374,7 @@
         <v>0.53650509859435258</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A84">
         <v>5</v>
       </c>
@@ -5409,7 +5409,7 @@
         <v>0.57053943574428556</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A85">
         <v>5</v>
       </c>
@@ -5444,7 +5444,7 @@
         <v>0.53980642235837872</v>
       </c>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A86">
         <v>5</v>
       </c>
@@ -5479,7 +5479,7 @@
         <v>0.54154368843883272</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A87">
         <v>5</v>
       </c>
@@ -5514,7 +5514,7 @@
         <v>0.54099914110265668</v>
       </c>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A88">
         <v>5</v>
       </c>
@@ -5549,7 +5549,7 @@
         <v>0.53899900997057559</v>
       </c>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A89">
         <v>5</v>
       </c>
@@ -5584,7 +5584,7 @@
         <v>0.54823849475942554</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A90">
         <v>5</v>
       </c>
@@ -5619,7 +5619,7 @@
         <v>0.53966674180701379</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A91">
         <v>6</v>
       </c>
@@ -5654,7 +5654,7 @@
         <v>0.1996115926653147</v>
       </c>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A92">
         <v>6</v>
       </c>
@@ -5689,7 +5689,7 @@
         <v>0.20157709019258621</v>
       </c>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A93">
         <v>6</v>
       </c>
@@ -5724,7 +5724,7 @@
         <v>0.20433659404516219</v>
       </c>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A94">
         <v>6</v>
       </c>
@@ -5759,7 +5759,7 @@
         <v>0.20724731064401569</v>
       </c>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A95">
         <v>6</v>
       </c>
@@ -5794,7 +5794,7 @@
         <v>0.20426760804839431</v>
       </c>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A96">
         <v>6</v>
       </c>
@@ -5829,7 +5829,7 @@
         <v>0.20419440823607149</v>
       </c>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A97">
         <v>6</v>
       </c>
@@ -5864,7 +5864,7 @@
         <v>0.2024935705587268</v>
       </c>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A98">
         <v>6</v>
       </c>
@@ -5899,7 +5899,7 @@
         <v>0.20528086428530509</v>
       </c>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A99">
         <v>7</v>
       </c>
@@ -5934,7 +5934,7 @@
         <v>0.30799950337968768</v>
       </c>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A100">
         <v>7</v>
       </c>
@@ -5969,7 +5969,7 @@
         <v>0.30740295867435641</v>
       </c>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A101">
         <v>7</v>
       </c>
@@ -6004,7 +6004,7 @@
         <v>0.30910372082144022</v>
       </c>
     </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A102">
         <v>7</v>
       </c>
@@ -6039,7 +6039,7 @@
         <v>0.30662859659641978</v>
       </c>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A103">
         <v>7</v>
       </c>
@@ -6074,7 +6074,7 @@
         <v>0.30936323581263431</v>
       </c>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A104">
         <v>7</v>
       </c>
@@ -6109,7 +6109,7 @@
         <v>0.30731362053193151</v>
       </c>
     </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A105">
         <v>7</v>
       </c>
@@ -6144,7 +6144,7 @@
         <v>0.30809800913557411</v>
       </c>
     </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A106">
         <v>7</v>
       </c>
@@ -6179,7 +6179,7 @@
         <v>0.31001204680651429</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A107">
         <v>7</v>
       </c>
@@ -6214,7 +6214,7 @@
         <v>0.30857269819825889</v>
       </c>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A108">
         <v>7</v>
       </c>
@@ -6249,7 +6249,7 @@
         <v>0.30571095142513521</v>
       </c>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A109">
         <v>7</v>
       </c>
@@ -6284,7 +6284,7 @@
         <v>0.31162585462443532</v>
       </c>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A110">
         <v>7</v>
       </c>
@@ -6319,7 +6319,7 @@
         <v>0.30607132334262133</v>
       </c>
     </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A111">
         <v>7</v>
       </c>
@@ -6354,7 +6354,7 @@
         <v>0.3114406032022089</v>
       </c>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A112">
         <v>7</v>
       </c>
@@ -6389,7 +6389,7 @@
         <v>0.30812599775381389</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A113">
         <v>7</v>
       </c>
@@ -6424,7 +6424,7 @@
         <v>0.30636434298940002</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A114">
         <v>7</v>
       </c>
@@ -6459,7 +6459,7 @@
         <v>0.32235423945821817</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A115">
         <v>8</v>
       </c>
@@ -6494,7 +6494,7 @@
         <v>55.250419767433783</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A116">
         <v>8</v>
       </c>
@@ -6529,7 +6529,7 @@
         <v>55.449371733749288</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A117">
         <v>8</v>
       </c>
@@ -6564,7 +6564,7 @@
         <v>55.262224439578127</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A118">
         <v>8</v>
       </c>
@@ -6599,7 +6599,7 @@
         <v>55.529484652355308</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A119">
         <v>8</v>
       </c>
@@ -6634,7 +6634,7 @@
         <v>55.32661248669028</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A120">
         <v>8</v>
       </c>
@@ -6669,7 +6669,7 @@
         <v>55.744315328774967</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A121">
         <v>8</v>
       </c>
@@ -6704,7 +6704,7 @@
         <v>55.109144209418453</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A122">
         <v>8</v>
       </c>
@@ -6739,7 +6739,7 @@
         <v>55.34271600181237</v>
       </c>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A123">
         <v>9</v>
       </c>
@@ -6774,7 +6774,7 @@
         <v>2.7405037511605772</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A124">
         <v>9</v>
       </c>
@@ -6809,7 +6809,7 @@
         <v>2.745556110516191</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A125">
         <v>9</v>
       </c>
@@ -6844,7 +6844,7 @@
         <v>2.7347435072064399</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A126">
         <v>9</v>
       </c>
@@ -6879,7 +6879,7 @@
         <v>2.733886868692935</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A127">
         <v>9</v>
       </c>
@@ -6914,7 +6914,7 @@
         <v>2.7477678807917978</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A128">
         <v>9</v>
       </c>
@@ -6949,7 +6949,7 @@
         <v>2.7346450057346372</v>
       </c>
     </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A129">
         <v>9</v>
       </c>
@@ -6984,7 +6984,7 @@
         <v>2.7386064060032371</v>
       </c>
     </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A130">
         <v>9</v>
       </c>
@@ -7019,7 +7019,7 @@
         <v>2.7680488591548049</v>
       </c>
     </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A131">
         <v>10</v>
       </c>
@@ -7054,7 +7054,7 @@
         <v>0.1030845830217004</v>
       </c>
     </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A132">
         <v>10</v>
       </c>
@@ -7089,7 +7089,7 @@
         <v>0.1028286766260862</v>
       </c>
     </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A133">
         <v>10</v>
       </c>
@@ -7124,7 +7124,7 @@
         <v>0.10300954654812811</v>
       </c>
     </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A134">
         <v>10</v>
       </c>
@@ -7159,7 +7159,7 @@
         <v>0.10330063798464829</v>
       </c>
     </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A135">
         <v>10</v>
       </c>
@@ -7194,7 +7194,7 @@
         <v>0.10042722262442109</v>
       </c>
     </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A136">
         <v>10</v>
       </c>
@@ -7229,7 +7229,7 @@
         <v>0.1026434725616127</v>
       </c>
     </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A137">
         <v>10</v>
       </c>
@@ -7264,7 +7264,7 @@
         <v>0.1051730264443904</v>
       </c>
     </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A138">
         <v>10</v>
       </c>
@@ -7299,7 +7299,7 @@
         <v>0.1030330980662257</v>
       </c>
     </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A139">
         <v>11</v>
       </c>
@@ -7334,7 +7334,7 @@
         <v>9.4313428787514564</v>
       </c>
     </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A140">
         <v>11</v>
       </c>
@@ -7369,7 +7369,7 @@
         <v>9.4611818093806512</v>
       </c>
     </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A141">
         <v>11</v>
       </c>
@@ -7404,7 +7404,7 @@
         <v>9.3503724219743169</v>
       </c>
     </row>
-    <row r="142" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A142">
         <v>11</v>
       </c>
@@ -7439,7 +7439,7 @@
         <v>9.4073665639851249</v>
       </c>
     </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A143">
         <v>11</v>
       </c>
@@ -7474,7 +7474,7 @@
         <v>25.137761257169771</v>
       </c>
     </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A144">
         <v>11</v>
       </c>
@@ -7509,7 +7509,7 @@
         <v>24.816892843041568</v>
       </c>
     </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A145">
         <v>11</v>
       </c>
@@ -7544,7 +7544,7 @@
         <v>24.858018419658769</v>
       </c>
     </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A146">
         <v>11</v>
       </c>
@@ -7579,7 +7579,7 @@
         <v>24.99993094420061</v>
       </c>
     </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A147">
         <v>11</v>
       </c>
@@ -7614,7 +7614,7 @@
         <v>24.855100932810451</v>
       </c>
     </row>
-    <row r="148" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A148">
         <v>11</v>
       </c>
@@ -7649,7 +7649,7 @@
         <v>24.800206984020772</v>
       </c>
     </row>
-    <row r="149" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A149">
         <v>11</v>
       </c>
@@ -7684,7 +7684,7 @@
         <v>24.618350029969591</v>
       </c>
     </row>
-    <row r="150" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A150">
         <v>11</v>
       </c>
@@ -7719,7 +7719,7 @@
         <v>25.04988603023812</v>
       </c>
     </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A151">
         <v>12</v>
       </c>
@@ -7754,7 +7754,7 @@
         <v>0.77132530906237662</v>
       </c>
     </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A152">
         <v>12</v>
       </c>
@@ -7789,7 +7789,7 @@
         <v>0.76786580076441169</v>
       </c>
     </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A153">
         <v>12</v>
       </c>
@@ -7824,7 +7824,7 @@
         <v>0.75745269376784563</v>
       </c>
     </row>
-    <row r="154" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A154">
         <v>12</v>
       </c>
@@ -7859,7 +7859,7 @@
         <v>0.77642538286745544</v>
       </c>
     </row>
-    <row r="155" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A155">
         <v>12</v>
       </c>
@@ -7894,7 +7894,7 @@
         <v>1.8744755972642451</v>
       </c>
     </row>
-    <row r="156" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A156">
         <v>12</v>
       </c>
@@ -7929,7 +7929,7 @@
         <v>1.9118938693311061</v>
       </c>
     </row>
-    <row r="157" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A157">
         <v>12</v>
       </c>
@@ -7964,7 +7964,7 @@
         <v>1.9222090917173771</v>
       </c>
     </row>
-    <row r="158" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A158">
         <v>12</v>
       </c>
@@ -7999,7 +7999,7 @@
         <v>1.9296134959906339</v>
       </c>
     </row>
-    <row r="159" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A159">
         <v>12</v>
       </c>
@@ -8034,7 +8034,7 @@
         <v>1.9297395583707839</v>
       </c>
     </row>
-    <row r="160" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A160">
         <v>12</v>
       </c>
@@ -8069,7 +8069,7 @@
         <v>1.9641987405717369</v>
       </c>
     </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A161">
         <v>12</v>
       </c>
@@ -8104,7 +8104,7 @@
         <v>1.919601474795491</v>
       </c>
     </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A162">
         <v>12</v>
       </c>
@@ -8139,7 +8139,7 @@
         <v>1.881445601629093</v>
       </c>
     </row>
-    <row r="165" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:11" x14ac:dyDescent="0.45">
       <c r="F165" s="3" t="s">
         <v>165</v>
       </c>
@@ -8159,7 +8159,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="166" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:11" x14ac:dyDescent="0.45">
       <c r="E166" s="1" t="s">
         <v>170</v>
       </c>
@@ -8188,7 +8188,7 @@
         <v>6.4987004749207316</v>
       </c>
     </row>
-    <row r="167" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:11" x14ac:dyDescent="0.45">
       <c r="E167" s="1" t="s">
         <v>171</v>
       </c>

</xml_diff>